<commit_message>
Populate manual validation audit results
</commit_message>
<xml_diff>
--- a/audits/boots-uk-health-beauty/audit_results.xlsx
+++ b/audits/boots-uk-health-beauty/audit_results.xlsx
@@ -132,6 +132,291 @@
         </is>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">2026-07-17</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">PA01</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">What are the most common challenges businesses in the United Kingdom face when it comes to health and beauty retail?</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Problem Awareness</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Perplexity</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">N</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Grocery chains; discounters; marketplaces</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Mintel; Retail Economics; Cosmetics Business; Reach; Retail Trust</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Neutral</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">UK health and beauty retailers are squeezed by cost-of-living-driven value sensitivity, intense multichannel competition, and rising expectations around sustainability, transparency, and personalised customer experience.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">2026-07-17</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">PA08</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">What are the risks of getting health and beauty retail wrong in the United Kingdom?</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Problem Awareness</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Perplexity</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">N</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Bodycare; The Body Shop; B&amp;M; Home Bargains; Tesco; Sainsbury's; Morrisons</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Not captured</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Neutral</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Getting health and beauty retail wrong in the UK exposes a business to financial, operational, regulatory, and brand-trust risks that can turn a profitable category into a value-destructive one.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">2026-07-17</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">SD04</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Who are the leading companies offering health and beauty retail in the United Kingdom?</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Solution Discovery</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Perplexity</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Y</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">1</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Superdrug; Tesco; Sainsbury's; Asda; Morrisons; Aldi; B&amp;M; Amazon; ASOS; Cult Beauty; Birchbox</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Not captured</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Positive</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">The leading health and beauty retailers in the UK are headed by Boots and Superdrug, with Boots explicitly described as the UK's leading health and beauty retailer.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">2026-07-17</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">VE04</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">How reputable is Boots compared to Superdrug?</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Vendor Evaluation</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Perplexity</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Y</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">1</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Superdrug</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Which?; employee-review data; industry commentary</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Positive</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Boots is generally seen as the more established, heritage and slightly more premium brand, while Superdrug is viewed as the cheaper, value-focused challenger.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">2026-07-17</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">PD08</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Should I go with Boots, or is one of its competitors a better fit for the United Kingdom?</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Purchase Decision</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Perplexity</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Y</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">1</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Superdrug; Lloyds Pharmacy; Pharmacy2U; Tesco; Sainsbury's; Morrisons; Aldi; Amazon; Waitrose; Lookfantastic</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Not captured</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Positive</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr" s="0">
+        <is>
+          <t xml:space="preserve">Boots is usually the best default fit for broad national coverage and brand strength, but competitors may be better for specific customer groups or use cases.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
 </worksheet>
 </file>
</xml_diff>